<commit_message>
Ejecución semanal 2026-S38: Esther Busso (Ajuntament de Castelló d'Empúries)
Lote de 25 municipios (Tenerife/La Gomera/La Palma + norte de Girona).
Búsqueda agrupada por dominios (tenerife.es excluido por ser del Cabildo):
1 contacto válido con email verificado, verificada su correspondencia con
la fila Castelló d'Empúries/Girona de la BBDD. Sin descartes. 1 crédito.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K228"/>
+  <dimension ref="A1:K229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10536,6 +10536,63 @@
       <c r="K228" s="2" t="inlineStr">
         <is>
           <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>Castelló d'Empúries</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Esther</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>Busso</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>Auxiliar Técnico de Medio Ambiente</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>ebusso@castello.cat</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/esther-bussó-66b6a231</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -10606,7 +10663,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7">
@@ -10616,7 +10673,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -10631,7 +10688,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registrar rebotes de la campaña y devolver esos municipios a la rotación
12 direcciones fallaron en la primera semana de envíos (10 rebotes + 2 en
la lista negra global de Apollo). Se marcan en la columna nueva
estado_email del CSV y del Excel, y dejan de contar como email válido, de
modo que el agente vuelva a buscar contacto en esos municipios.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K229"/>
+  <dimension ref="A1:L229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -437,6 +437,7 @@
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,6 +496,11 @@
           <t>Fecha alta</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Estado del email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -540,6 +546,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -585,6 +592,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -630,6 +638,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -675,6 +684,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -720,6 +730,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -765,6 +776,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -810,6 +822,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -855,6 +868,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -900,6 +914,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -945,6 +960,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -990,6 +1006,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1035,6 +1052,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1080,6 +1098,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1125,6 +1144,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1170,6 +1190,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1215,6 +1236,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1260,6 +1282,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1305,6 +1328,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1350,6 +1374,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1395,6 +1420,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1440,6 +1470,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1481,6 +1512,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1526,6 +1558,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1571,6 +1604,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1616,6 +1650,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1661,6 +1696,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1706,6 +1742,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1747,6 +1784,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1792,6 +1830,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1837,6 +1876,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1878,6 +1918,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1923,6 +1964,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1968,6 +2010,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2009,6 +2052,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2050,6 +2094,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2095,6 +2140,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2136,6 +2182,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2181,6 +2228,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2222,6 +2270,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2267,6 +2316,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2312,6 +2362,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2357,6 +2408,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2402,6 +2454,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2447,6 +2500,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2492,6 +2546,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2537,6 +2592,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2582,6 +2638,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2627,6 +2684,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2672,6 +2730,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2717,6 +2776,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2762,6 +2822,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2807,6 +2868,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2852,6 +2914,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2897,6 +2960,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2942,6 +3006,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2987,6 +3052,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3032,6 +3098,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3077,6 +3144,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3122,6 +3190,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3167,6 +3236,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3212,6 +3282,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3257,6 +3328,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3302,6 +3374,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3347,6 +3420,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3392,6 +3466,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3437,6 +3512,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3482,6 +3558,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3527,6 +3604,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3572,6 +3654,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3617,6 +3700,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3662,6 +3746,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3707,6 +3792,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3752,6 +3838,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3797,6 +3884,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3842,6 +3930,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3887,6 +3976,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3932,6 +4022,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3977,6 +4068,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4022,6 +4118,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4067,6 +4164,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4112,6 +4210,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4157,6 +4256,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4202,6 +4302,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4247,6 +4348,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4292,6 +4394,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4337,6 +4440,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4382,6 +4486,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4427,6 +4532,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4472,6 +4578,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4517,6 +4624,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4562,6 +4670,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4607,6 +4720,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4652,6 +4766,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4697,6 +4812,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4742,6 +4858,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4787,6 +4904,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4832,6 +4950,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4877,6 +4996,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4922,6 +5042,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4967,6 +5088,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5012,6 +5134,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5057,6 +5180,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5102,6 +5226,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5147,6 +5272,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5192,6 +5318,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5237,6 +5364,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5282,6 +5410,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -5327,6 +5456,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5372,6 +5502,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -5417,6 +5548,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5462,6 +5598,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5507,6 +5644,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5552,6 +5690,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5593,6 +5732,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L115" s="2" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5638,6 +5778,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5683,6 +5824,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5728,6 +5870,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -5773,6 +5916,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5818,6 +5962,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -5863,6 +6012,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5908,6 +6058,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -5953,6 +6104,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L123" s="2" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5998,6 +6150,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -6043,6 +6196,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L125" s="2" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -6088,6 +6242,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -6133,6 +6288,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L127" s="2" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6174,6 +6330,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6215,6 +6372,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L129" s="2" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6260,6 +6418,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -6305,6 +6464,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L131" s="2" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6346,6 +6506,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -6389,6 +6550,11 @@
       <c r="K133" s="2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>lista negra Apollo</t>
         </is>
       </c>
     </row>
@@ -6432,6 +6598,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -6473,6 +6640,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6514,6 +6682,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -6555,6 +6724,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -6596,6 +6766,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -6637,6 +6808,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L139" s="2" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -6682,6 +6854,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -6727,6 +6904,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -6772,6 +6950,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -6817,6 +6996,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6862,6 +7042,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -6907,6 +7088,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6952,6 +7138,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -6997,6 +7184,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>lista negra Apollo</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -7042,6 +7234,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -7087,6 +7280,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -7132,6 +7326,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -7177,6 +7372,11 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -7222,6 +7422,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -7263,6 +7464,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -7304,6 +7506,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -7345,6 +7548,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -7386,6 +7590,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -7427,6 +7632,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -7472,6 +7678,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L158" s="2" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -7517,6 +7724,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L159" s="2" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -7558,6 +7766,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -7599,6 +7808,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -7640,6 +7850,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -7685,6 +7896,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L163" s="2" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -7726,6 +7938,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L164" s="2" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -7771,6 +7984,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L165" s="2" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -7816,6 +8030,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -7857,6 +8072,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L167" s="2" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -7902,6 +8118,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L168" s="2" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -7943,6 +8160,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L169" s="2" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -7984,6 +8202,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L170" s="2" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -8025,6 +8244,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L171" s="2" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -8066,6 +8286,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L172" s="2" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -8111,6 +8332,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L173" s="2" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -8152,6 +8374,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L174" s="2" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -8193,6 +8416,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L175" s="2" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -8238,6 +8462,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L176" s="2" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -8279,6 +8504,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L177" s="2" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -8320,6 +8546,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L178" s="2" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -8361,6 +8588,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L179" s="2" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -8406,6 +8634,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L180" s="2" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -8447,6 +8676,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L181" s="2" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -8488,6 +8718,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -8529,6 +8760,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L183" s="2" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -8570,6 +8802,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L184" s="2" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -8611,6 +8844,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L185" s="2" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -8656,6 +8890,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L186" s="2" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -8697,6 +8932,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L187" s="2" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -8738,6 +8974,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L188" s="2" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -8779,6 +9016,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L189" s="2" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -8824,6 +9062,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L190" s="2" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -8869,6 +9108,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L191" s="2" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -8914,6 +9154,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L192" s="2" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -8959,6 +9200,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L193" s="2" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -9004,6 +9246,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L194" s="2" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -9045,6 +9288,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L195" s="2" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -9086,6 +9330,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L196" s="2" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -9131,6 +9376,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L197" s="2" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -9172,6 +9418,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L198" s="2" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -9213,6 +9460,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L199" s="2" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -9254,6 +9502,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L200" s="2" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -9295,6 +9544,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L201" s="2" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -9336,6 +9586,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L202" s="2" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -9381,6 +9632,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L203" s="2" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -9426,6 +9678,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L204" s="2" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -9467,6 +9720,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L205" s="2" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -9512,6 +9766,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L206" s="2" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -9557,6 +9812,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L207" s="2" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -9602,6 +9858,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L208" s="2" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -9647,6 +9904,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L209" s="2" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -9692,6 +9950,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L210" s="2" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -9737,6 +9996,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L211" s="2" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -9782,6 +10042,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L212" s="2" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -9827,6 +10088,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L213" s="2" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -9872,6 +10134,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L214" s="2" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -9917,6 +10180,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L215" s="2" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -9958,6 +10222,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L216" s="2" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -10003,6 +10268,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L217" s="2" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -10048,6 +10314,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L218" s="2" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -10089,6 +10356,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L219" s="2" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -10130,6 +10398,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L220" s="2" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -10175,6 +10444,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L221" s="2" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -10220,6 +10490,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L222" s="2" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -10265,6 +10536,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L223" s="2" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -10310,6 +10582,7 @@
           <t>2026-09-01</t>
         </is>
       </c>
+      <c r="L224" s="2" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -10367,6 +10640,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L225" s="2" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -10424,6 +10698,11 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L226" s="2" t="inlineStr">
+        <is>
+          <t>rebotado 09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -10481,6 +10760,7 @@
           <t>2026-09-02</t>
         </is>
       </c>
+      <c r="L227" s="2" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -10538,6 +10818,7 @@
           <t>2026-09-07</t>
         </is>
       </c>
+      <c r="L228" s="2" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -10595,6 +10876,7 @@
           <t>2026-09-14</t>
         </is>
       </c>
+      <c r="L229" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10607,7 +10889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -10643,7 +10925,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>172</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5">
@@ -10653,7 +10935,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -10663,32 +10945,42 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>173</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>Emails rebotados o en lista negra</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>Contactos nominales (Apollo)</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B8" s="2" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-    </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Última actualización del agente</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ejecución semanal 2026-S39: 3 contactos nuevos en el Baix Empordà
Pere Bofill (Sant Feliu de Guíxols), Susa Bonilla (Calonge i Sant Antoni)
y Rut Palomeque (Palafrugell), los tres técnicos de medio ambiente con
email verificado y municipio/provincia verificados. Añadidos a la lista,
a HubSpot e inscritos en la secuencia (que está pausada a mano, así que
quedan en espera). Créditos gastados: 3.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L229"/>
+  <dimension ref="A1:L232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -10877,6 +10877,180 @@
         </is>
       </c>
       <c r="L229" s="2" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>Sant Feliu de Guíxols</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Pere</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>Bofill Arbusa</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>Tècnic de Medi Ambient</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>pbofill@guixols.cat</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/pere-bofill-arbusà-3913b646</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>Calonge i Sant Antoni</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Susa</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>Bonilla</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>Tècnica de Medi Ambient, Parcs i Jardins</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>susa.bonilla@calonge.cat</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/susa-bonilla-b928b9a4</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="L231" s="2" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>Palafrugell</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>Girona</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>Rut</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>Palomeque</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>Tècnica de Medi Ambient</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>rpalomeque@palafrugell.net</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/rut-palomeque-2042778b</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K232" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="L232" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10945,7 +11119,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7">
@@ -10965,7 +11139,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Recuperar las pasadas del 28/09 y del 12/10 en la base de datos
Las dos pasadas dieron de alta sus contactos en Apollo, pero el commit del
CSV y de state.json se perdió al reciclarse el contenedor a mitad de
ejecución. Al no avanzar state.json, el lote del 12/10 volvió a salir con
los mismos 25 municipios del 28/09.

Se añaden las 13 filas que faltaban (5 del 28/09 + 8 del 12/10), todas con
municipio y provincia copiados de su fila del CSV y comprobados fila a fila
antes de escribir, y se marcan los 25 municipios del lote como procesados
para que la rotación siga por Girona y Castellón.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015oaFpSagWroLdzsbC55cuL
</commit_message>
<xml_diff>
--- a/data/ayuntamientos-costeros.xlsx
+++ b/data/ayuntamientos-costeros.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L232"/>
+  <dimension ref="A1:L245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11051,6 +11051,760 @@
         </is>
       </c>
       <c r="L232" s="2" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>Castelldefels</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>Manu</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>Reyes</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>manuel.reyes@castelldefels.org</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I233" s="2" t="inlineStr">
+        <is>
+          <t>Apollo (búsqueda verificada)</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K233" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L233" s="2" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>Gavà</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>Jordi</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>Tort</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>Tinent d'Alcaldessa de Planificació Territorial i Medi Ambient</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>jtort@gava.cat</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>Apollo (búsqueda verificada)</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K234" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L234" s="2" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>Vilanova i la Geltrú</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>Ester</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>Tècnica de Medi Ambient</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>etoledo@vilanova.cat</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>Apollo (búsqueda verificada)</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K235" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L235" s="2" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>Salou</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>Eugeni</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>Capella Roca</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>Tècnic de Medi Ambient</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>ecapella@salou.cat</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>Apollo (búsqueda verificada)</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K236" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L236" s="2" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>Calafell</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>Ramon</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>Ferre</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>rferre@calafell.org</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>Apollo (búsqueda verificada)</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K237" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L237" s="2" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>El Prat de Llobregat</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>Perez Castro</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>Tinent d'Alcalde d'Acció Institucional, Projectes Urbans i Mobilitat</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>perezjp@elprat.cat</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/juanpedroperez</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K238" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L238" s="2" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>Premià de Mar</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>Jordi</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>Lluch</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>Cap de Servei de Medi Ambient, Salut Pública i Benestar Animal</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>lluchtj@premiademar.cat</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/jordi-lluch-73a8415</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K239" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L239" s="2" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>Mataró</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Toni</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>Merino</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>Gerente Municipal</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>amerino@ajmataro.cat</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/tonimerino</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K240" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L240" s="2" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>Sant Vicenç de Montalt</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>Rabat Fajardo</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>Auxiliar Administrativo en Regidoria de Urbanismo y Medio Ambiente</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>jrabat@svmontalt.cat</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/jrabatf</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K241" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L241" s="2" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>El Vendrell</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>Noelia</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>Gonzalez Sigueenza</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Arquitecta Urbanista</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>ngonzalez@elvendrell.net</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/noeliagonzalez-arquitecta</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L242" s="2" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>Torredembarra</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>Angie</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>Munoz</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Regidora de Sostenibilitat, Salubritat i Benestar Animal</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>a.munoz@torredembarra.cat</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/angie-mu%c3%b1oz-b592541b1</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Rut</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>Fabra</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Arquitecta en Serveis Tècnics d'Urbanisme</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>rfabra@tarragona.cat</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/rut-fabra-278b1a44</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K244" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L244" s="2" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>Vila-seca</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>Cristina</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>Cid</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>Concejala de Innovación y Servicios al Territorio</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>ccid@vila-seca.cat</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>Nominal (Apollo · verificado)</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>http://www.linkedin.com/in/cristina-c-cid-8986574a</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>apollo</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="L245" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11119,7 +11873,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7">
@@ -11139,7 +11893,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -11154,7 +11908,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>

</xml_diff>